<commit_message>
agent v7: measured tier confidence (A 11/11, B 24/24, C 3/5 on 43 hand checks), Excel, reports and results.zip from v7
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWAhyUcdYXqypsWJ8kvKA8
</commit_message>
<xml_diff>
--- a/agent/reports/metadaten_challenge_alle.xlsx
+++ b/agent/reports/metadaten_challenge_alle.xlsx
@@ -632,17 +632,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Spital Schwyz (Chronischkrankenhaus)</t>
+          <t>Alterszentrum Acherhof</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Grosser Mythen</t>
+          <t>Gross Mythen; Chli Mythen</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Waldeggstrasse 12</t>
+          <t>Grundstrasse 32a</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -651,43 +651,43 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>47.0155</v>
+        <v>47.018485</v>
       </c>
       <c r="K2" t="n">
-        <v>8.6595</v>
+        <v>8.656758</v>
       </c>
       <c r="L2" t="n">
-        <v>2692825</v>
+        <v>2692611</v>
       </c>
       <c r="M2" t="n">
-        <v>1207883</v>
+        <v>1208211</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0.6</v>
+        <v>0.962</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Geländeprüfung, Bildinhalt); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung). Zwei unabhängige Analysen nennen verschiedene Orte (Brunnen, Ingenbohl / Schwyz); Prüfung nötig.</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis setzt Waldeggstrasse 12 in die Ortschaft Schwyz (PLZ 6430). | Die Skyline von der Wiese südwestlich des Spitals zeigt den Grossen Mythen im Nordosten mit dem nach links abfallenden Grat, so wie im Foto. (https://api3.geo.admin.ch/rest/services/profile.json?geom=%7B%22type%22%3A%22LineString%22%2C%22coordinates%22%3A%5B%5B2692697%2C1207770%5D%2C%5B2695004%2C1209518%5D%5D%7D&amp;sr=2056&amp;nb_points=200) | Der Grosse Mythen von Süden gesehen rechts hinter dem Gebäude weist auf den Talkessel von Schwyz hin.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | swissNAMES3D (swisstopo)</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-10-23T23:12:15Z</t>
+          <t>2026-10-24T08:07:29Z</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Hotel Restaurant Alpstubli</t>
+          <t>Alpstubli</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -763,26 +763,26 @@
         <v>1203886</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Text im Bild, Karte); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt Ringstrasse 111 in der Ortschaft Stoos SZ (PLZ 6433). | In OSM ist das Restaurant Alpstubli an der Ringstrasse 111 in Morschach (Stoos) verzeichnet. (https://www.openstreetmap.org/way/247158974) | Am Gebäude ist der Schriftzug «Alpstubli» zu lesen.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die Aufschrift «Alpstubli» steht auf einem grossen Hotelbau mit Terrasse an einem autofreien Weg. Das passt zum Hotel Alpstubli auf dem Stoos an der Ringstrasse 111 und nicht zum kleineren Alpstubli an der Ibergeregg.</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2026-10-23T23:07:41Z</t>
+          <t>2026-10-24T08:06:29Z</t>
         </is>
       </c>
     </row>
@@ -842,12 +842,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pfarrkirche St. Georg und Zeno; Aufbewahrungshalle (Bahnhofstrasse 8)</t>
+          <t>Pfarrkirche St. Georg und Zeno</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Rigi</t>
+          <t>Rigi Kulm</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -861,38 +861,38 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>47.06345</v>
+        <v>47.063491</v>
       </c>
       <c r="K4" t="n">
-        <v>8.52342</v>
+        <v>8.523220999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>2682405</v>
+        <v>2682390</v>
       </c>
       <c r="M4" t="n">
-        <v>1213061</v>
+        <v>1213065</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 4 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>Verifiziertes Referenzfoto (151 Inlier) zeigt die Pfarrkirche St. Georg und Zeno in Arth. (https://commons.wikimedia.org/wiki/File:Arth_Pfarrkirche_St._Georg_und_Zeno_5.jpg) | Referenzfoto 23 m entfernt zeigt dasselbe Kirchenschiff mit rotem Dachreiter aus fast gleichem Blickwinkel in Arth. (https://commons.wikimedia.org/wiki/File:Arth_Pfarrkirche_St._Georg_und_Zeno_6.jpg) | Amtliches Adressverzeichnis: Bahnhofstrasse 8/10 liegt in der Ortschaft Arth (6415).</t>
+          <t>Vergleichsfoto vor Ort: Arth Pfarrkirche St. Georg und Zeno 6 (37 m, 335 passende Punkte) (https://commons.wikimedia.org/wiki/File:Arth_Pfarrkirche_St._Georg_und_Zeno_6.jpg) | Vergleichsfoto vor Ort: Arth Pfarrkirche St. Georg und Zeno 5 (58 m, 151 passende Punkte) (https://commons.wikimedia.org/wiki/File:Arth_Pfarrkirche_St._Georg_und_Zeno_5.jpg) | Bildsuche: Arth Pfarrkirche St. Georg und Zeno 6 (335 passende Punkte) (https://commons.wikimedia.org/wiki/File:Arth_Pfarrkirche_St._Georg_und_Zeno_6.jpg)</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2026-10-23T23:09:27Z</t>
+          <t>2026-10-24T08:06:50Z</t>
         </is>
       </c>
     </row>
@@ -935,64 +935,37 @@
       <c r="C5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Morschach</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Morschach</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Urirotstock</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>31.12.2004</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>46.9822</v>
-      </c>
-      <c r="K5" t="n">
-        <v>8.6165</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2689611</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1204131</v>
-      </c>
       <c r="N5" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Geländeprüfung, Bildinhalt, Gebäudeadressverzeichnis); Gemeinde durch 3 unabhängige Quellen gestützt (Geländeprüfung, Bildinhalt, Gebäudeadressverzeichnis); Gebäude, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe -: Kein belastbarer Hinweis auf den Ort: offen gelassen. Konfidenz: Schätzwert, noch nicht gemessen.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Gebäude, Strasse</t>
+          <t>Ortschaft, Gemeinde, Gebäude, See/Fluss/Berg, Strasse</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
@@ -1005,11 +978,6 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Die Skyline-Berechnung von Morschach Richtung Süden zeigt ein ähnliches Profil wie das Bergmassiv im Bild, bei Gegenlicht passend zum Sonnenstand. | Ein hochgelegener Hotelbau mit Blick über ein dunstiges Tal auf ein vergletschertes Massiv passt zur Lage von Morschach über dem Urnersee. | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Morschach).</t>
-        </is>
-      </c>
       <c r="Y5" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1017,7 +985,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-10-23T23:17:25Z</t>
+          <t>2026-10-24T08:06:47Z</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1020,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Vierwaldstättersee; Urmiberg</t>
+          <t>Brunnen-Urmiberg; Urnersee; Vierwaldstättersee</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Gersauerstrasse</t>
+          <t>Gersauerstrasse 91</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1066,38 +1034,38 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>47.0005</v>
+        <v>47.000269</v>
       </c>
       <c r="K6" t="n">
-        <v>8.580500000000001</v>
+        <v>8.580225</v>
       </c>
       <c r="L6" t="n">
-        <v>2686843</v>
+        <v>2686822</v>
       </c>
       <c r="M6" t="n">
-        <v>1206125</v>
+        <v>1206099</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1112,7 +1080,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet den Hafenpunkt der Ortschaft Brunnen (6440) zu. | OSM führt den Hafen als 'Marina Fallenbach Brunnen'. (https://www.openstreetmap.org/way/1074836664) | Das Session-Foto zeigt die Urmiberg-Seilbahn über Brunnen; der Hafen liegt am Fuss des Urmibergs.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Das Serienfoto zeigt die Luftseilbahn Brunnen–Urmiberg mit Blick auf Brunnen und den Urnersee. Mit Tele aufgenommen sieht man von dort hinunter auf den grossen Jachthafen am Fuss des bewaldeten Urmiberg-Steilhangs. Das ist die Marina Fallenbach an der Gersauerstrasse mit Werft, Travellift und Slipanlage.</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1122,7 +1090,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-10-23T23:10:30Z</t>
+          <t>2026-10-24T08:07:09Z</t>
         </is>
       </c>
     </row>
@@ -1150,9 +1118,9 @@
           <t>Ingenbohl</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Kräuterhaus Rophaien</t>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Alte Kantonsstrasse 12</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1161,48 +1129,48 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>46.9958</v>
+        <v>46.999077</v>
       </c>
       <c r="K7" t="n">
-        <v>8.6075</v>
+        <v>8.611307</v>
       </c>
       <c r="L7" t="n">
-        <v>2688904</v>
+        <v>2689188</v>
       </c>
       <c r="M7" t="n">
-        <v>1205633</v>
+        <v>1206001</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0</v>
+        <v>0.962</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Text im Bild, Gebäudeadressverzeichnis); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Text im Bild); See/Fluss/Berg, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>See/Fluss/Berg, Strasse</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Gebäude, See/Fluss/Berg</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1212,7 +1180,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Die Fassadeninschrift „Kräuterhaus Rophaien Herboristerie“ nennt die Kräuterfirma Rophaien, die nach eigenem Wissen ihren Sitz in 6440 Brunnen hat. | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Brunnen). | Laut amtlichem Ortschaftenverzeichnis gehört die Ortschaft Brunnen (6440) zur Gemeinde Ingenbohl.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die Fassadenschrift «Kräuterhaus Rophaien Herboristerie» ist zu lesen; laut Presse steht das Kräuterhaus Rophaien an der Alten Kantonsstrasse 12 in Brunnen, und das Adressregister bestätigt diese Adresse.</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1222,7 +1190,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-10-23T23:11:45Z</t>
+          <t>2026-10-24T08:07:12Z</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1220,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Kapelle 14 Nothelfer (Nothelferkapelle)</t>
+          <t>Nothelferkapelle</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1278,26 +1246,26 @@
         <v>1205505</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="Q8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1317,7 +1285,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Ein verifizierter Referenztreffer zeigt dieselbe Kapelle 14 Nothelfer in Brunnen (Gemeinde Ingenbohl). (https://commons.wikimedia.org/wiki/File:Kapelle_14_Nothelfer.jpg) | Ein zweiter verifizierter Treffer zeigt die Alte Gasse mit der Kapelle 14 Nothelfer in Brunnen. (https://commons.wikimedia.org/wiki/File:Alte_Gasse_mit_Kapelle_14_Nothelfer.jpg) | Laut amtlichem Adressverzeichnis liegt der Standort in der Ortschaft Brunnen (PLZ 6440).</t>
+          <t>Vergleichsfoto vor Ort: Kapelle 14 Nothelfer (9 m, 139 passende Punkte) (https://commons.wikimedia.org/wiki/File:Kapelle_14_Nothelfer.jpg) | Bildsuche: Kapelle 14 Nothelfer (139 passende Punkte) (https://commons.wikimedia.org/wiki/File:Kapelle_14_Nothelfer.jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1327,7 +1295,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-10-23T23:12:04Z</t>
+          <t>2026-10-24T08:07:16Z</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1325,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Hotel du Lac Seehof</t>
+          <t>du Lac Seehof</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1371,38 +1339,38 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>47.08025</v>
+        <v>47.080204</v>
       </c>
       <c r="K9" t="n">
-        <v>8.439249999999999</v>
+        <v>8.439164999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>2675988</v>
+        <v>2675981</v>
       </c>
       <c r="M9" t="n">
-        <v>1214844</v>
+        <v>1214839</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Text im Bild, Gebäuderegister (OSM/GWR), Gebäudeadressverzeichnis); Gemeinde durch 3 unabhängige Quellen gestützt (Text im Bild, Gebäuderegister (OSM/GWR), Gebäudeadressverzeichnis); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1422,7 +1390,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Der Schriftzug «HOTEL du LAC SEEHOF» an der Fassade nennt das Hotel am Seeplatz in Küssnacht. | OSM führt das Hotel «du Lac Seehof» am Seeplatz in Küssnacht (SZ). (https://www.openstreetmap.org/node/1411264386) | Das amtliche Adressverzeichnis gibt beim Hotel Seeplatz 6, 6403 Küssnacht am Rigi, an.</t>
+          <t>Vergleichsfoto vor Ort: Mapillary Küssnacht (SZ) 2018-08-29 (78 m, 60 passende Punkte) (https://www.mapillary.com/app/?pKey=2816197491926484) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1432,7 +1400,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>2026-10-23T23:12:54Z</t>
+          <t>2026-10-24T08:07:34Z</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1430,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Gipfelrestaurant Fronalpstock; Bergstation Sessellift Fronalpstock (2. Sektion)</t>
+          <t>Fronalpstock</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Fronalpstock</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1476,48 +1449,43 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>46.96975</v>
+        <v>46.969836</v>
       </c>
       <c r="K10" t="n">
-        <v>8.637079999999999</v>
+        <v>8.637148</v>
       </c>
       <c r="L10" t="n">
-        <v>2691198</v>
+        <v>2691203</v>
       </c>
       <c r="M10" t="n">
-        <v>1202771</v>
+        <v>1202781</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.6</v>
+        <v>0.962</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte); See/Fluss/Berg nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Stoos SZ, Morschach / Unteriberg, Schwyz); Prüfung nötig.</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>See/Fluss/Berg</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1527,7 +1495,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet Fronalpstock 1 der Ortschaft Stoos SZ (6433) zu. | Das GWR führt die Bergstation Sessellift 2. Sektion (Fronalpstock 2) in der Ortschaft Stoos SZ. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190289668_0) | Das Luftbild 2005 zeigt die gelbe Stationshaube direkt neben dem Restaurant und den Mast östlich davon, wie auf dem Foto.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Neuer Holzbau mit verglastem Saal und Terrasse auf einer Gipfelkuppe, direkt neben der gelben Bergstation einer Sesselbahn. Das passt zum Gipfelrestaurant Fronalpstock auf dem Stoos, das neben der Bergstation der Sesselbahn liegt.</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1537,7 +1505,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>2026-10-23T23:17:46Z</t>
+          <t>2026-10-24T08:07:35Z</t>
         </is>
       </c>
     </row>
@@ -1567,17 +1535,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Burgruine Schwanau; Restaurant Schwanau; Kapelle Schwanau</t>
+          <t>Burg Schwanau, mittelalterliche Burgruine</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Insel Schwanau; Lauerzersee</t>
+          <t>Lauerzersee</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Insel Schwanau 1a</t>
+          <t>Schwanau 1d</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1586,38 +1554,38 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>47.03245</v>
+        <v>47.032494</v>
       </c>
       <c r="K11" t="n">
-        <v>8.597300000000001</v>
+        <v>8.597434</v>
       </c>
       <c r="L11" t="n">
-        <v>2688068</v>
+        <v>2688078</v>
       </c>
       <c r="M11" t="n">
-        <v>1209695</v>
+        <v>1209700</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>1</v>
+        <v>0.962</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Gebäuderegister (OSM/GWR), Session-Foto); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Gebäuderegister (OSM/GWR), Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1632,7 +1600,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt die Insel Schwanau 1a in der Ortschaft 6424 Lauerz. | Die verifizierte Archivaufnahme 'Insel Schwanau im Winter' (Lauerz) zeigt dieselben Bauten. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=640332) | OSM führt die Burgruine, die Kapelle und das Restaurant Schwanau in Lauerz. (https://www.openstreetmap.org/relation/15976459)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Den Turm der Burgruine mit der Schwyzer Flagge, das Restaurant mit Flammenläden und die Kapelle mit dem roten Zwiebeltürmchen erkennt man eindeutig als Insel Schwanau. Auch das Serienfoto zeigt die Insel im Lauerzersee.</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1642,7 +1610,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2026-10-23T23:17:39Z</t>
+          <t>2026-10-24T08:07:39Z</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1645,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Grosser Mythen</t>
+          <t>Gross Mythen</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1703,26 +1671,26 @@
         <v>1211471</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1737,7 +1705,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Verifiziertes Referenzbild aus Steinen zeigt dieselbe Kapelle. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=360529) | Amtliches Adressverzeichnis: Ortschaft Steinen (6422) an der Kapelle. | OSM: Stauffacherkapelle in Steinen. (https://www.openstreetmap.org/way/205619472)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die Giebelinschrift über Stauffachers Haus von 1308 und das Steiner Wappen zeigen die Stauffacherkapelle an der Schwyzerstrasse in Steinen. Im Hintergrund sieht man Richtung Schwyz den Grossen Mythen.</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1747,7 +1715,7 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>2026-10-23T23:18:29Z</t>
+          <t>2026-10-24T08:07:51Z</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1745,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Hotel Schwert (Seeterrasse)</t>
+          <t>Schwert</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Vierwaldstättersee; Rigi</t>
+          <t>Rigi; Vierwaldstättersee</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Seestrasse 29</t>
+          <t>Seestrasse 28</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1796,38 +1764,38 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>46.99075</v>
+        <v>46.990773</v>
       </c>
       <c r="K13" t="n">
-        <v>8.5251</v>
+        <v>8.524908999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>2682645</v>
+        <v>2682630</v>
       </c>
       <c r="M13" t="n">
-        <v>1204981</v>
+        <v>1204984</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Text im Bild, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1842,7 +1810,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Die Aufschrift «Schwert Seeterrasse» am Gebäude passt zum Hotel Schwert in Gersau. | Laut swisstopo-Adressverzeichnis liegt der Standort in der Ortschaft Gersau (PLZ 6442). | OSM führt das Hotel Schwert in der Gemeinde Gersau am Seeufer. (https://www.openstreetmap.org/node/1586989752)</t>
+          <t>Vergleichsfoto vor Ort: Mapillary Gersau 2018-08-29 (51 m, 82 passende Punkte) (https://www.mapillary.com/app/?pKey=1124531408046974) | Bildsuche: Schifflände Gersau SZ (2014) (259 passende Punkte) (https://commons.wikimedia.org/wiki/File:Schiffl%C3%A4nde_Gersau_SZ_(2014).jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -1852,7 +1820,7 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>2026-10-23T23:18:20Z</t>
+          <t>2026-10-24T08:07:59Z</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1855,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Glattalp</t>
+          <t>Bisistal; Glattalpsee</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1913,26 +1881,26 @@
         <v>1197134</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Session-Foto); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Referenzfoto, Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1947,7 +1915,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet die Kapellenkoordinaten der Ortschaft Bisisthal (6436) zu. | Verifizierte Archivkarte 'Glattalp, Berggottesdienst vor der Glattalp-Kapelle, Bisisthal' zeigt dieselbe Kapelle. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=360340) | Session-Foto zeigt die Glattalphütte SAC in Bisisthal.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Eine kleine, mit Schindeln verkleidete Bergkapelle mit Festbänken steht an der Geländekante über einem tiefen Tal, ringsum liegt Schrattenkalk-Karst. Das Foto aus derselben Serie zeigt eine SAC-Hütte auf einem Hügel. Beides passt zur Glattalpkapelle bei der Bergstation, nahe der Glattalphütte SAC Mythen, über dem Bisistal.</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -1957,7 +1925,7 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>2026-10-23T23:18:22Z</t>
+          <t>2026-10-24T08:07:44Z</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1960,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Glattalp</t>
+          <t>Glattalpsee; Ortstock</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2006,38 +1974,38 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>46.91683</v>
+        <v>46.916773</v>
       </c>
       <c r="K15" t="n">
-        <v>8.87494</v>
+        <v>8.874853</v>
       </c>
       <c r="L15" t="n">
-        <v>2709404</v>
+        <v>2709397</v>
       </c>
       <c r="M15" t="n">
-        <v>1197193</v>
+        <v>1197186</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>0.5</v>
+        <v>0.923</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, swisstopo-Ortsname); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -2052,7 +2020,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis legt die Glattalphütte (Glattalp 3) in die Ortschaft Bisisthal, PLZ 6436. | Das Session-Foto zeigt die Glattalpkapelle (Glattalp 2, Bisisthal), die wenige hundert Meter neben der Hütte steht. | Laut swisstopo-Ortsverzeichnis liegt die Adresse Glattalp 3 in 6436 Bisisthal. (https://api3.geo.admin.ch/rest/services/api/SearchServer?searchText=Glattalp&amp;type=locations&amp;sr=2056&amp;limit=8)</t>
+          <t>Vergleichsfoto vor Ort: Glattalphütte September 2021 (47 m, 199 passende Punkte) (https://commons.wikimedia.org/wiki/File:Glattalph%C3%BCtte_September_2021.jpg) | Bildsuche: Glattalphütte September 2021 (199 passende Punkte) (https://commons.wikimedia.org/wiki/File:Glattalph%C3%BCtte_September_2021.jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -2062,7 +2030,7 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2026-10-23T23:21:54Z</t>
+          <t>2026-10-24T08:07:47Z</t>
         </is>
       </c>
     </row>
@@ -2080,19 +2048,14 @@
       <c r="C16" t="n">
         <v>1</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Arth</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Arth</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Goldauer Bergsturz; Gnipen; Rossberg; Lauerzersee; Rigi Hochflue</t>
+          <t>Fronalpstock; Gnipen; Gross Mythen; Chli Mythen; Lauerzersee; Rigiaa; Rossberg; Brunnen-Urmiberg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2101,43 +2064,43 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>47.0814</v>
+        <v>47.08176</v>
       </c>
       <c r="K16" t="n">
-        <v>8.5624</v>
+        <v>8.563152000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>2685338</v>
+        <v>2685394</v>
       </c>
       <c r="M16" t="n">
-        <v>1215098</v>
+        <v>1215139</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="R16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, swisstopo-Ortsname); Gemeinde durch 5 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, swisstopo-Ortsname, Session-Foto); Gebäude, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Gebäude, Strasse</t>
+          <t>Ortschaft, Gebäude, Strasse</t>
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr">
@@ -2152,7 +2115,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Laut amtlichem Ortschaftenverzeichnis liegt der Punkt beim Gnipen in der Ortschaft Arth (6415). | Verifiziertes Vergleichsbild «View onto the Goldauer Bergsturz» beim Gnipen, Gemeinde Arth. (https://commons.wikimedia.org/wiki/File:View_onto_the_Goldauer_Bergsturz_(14033656358).jpg) | swisstopo führt den Gipfel Gnipen in der Gemeinde Arth. (https://api3.geo.admin.ch/rest/services/api/SearchServer?searchText=Gnipen&amp;type=locations&amp;sr=2056&amp;limit=8)</t>
+          <t>Vergleichsfoto vor Ort: View onto the Goldauer Bergsturz (14033656358) (72 m, 214 passende Punkte) (https://commons.wikimedia.org/wiki/File:View_onto_the_Goldauer_Bergsturz_(14033656358).jpg) | Vergleichsfoto vor Ort: Goldauer Bergsturz (14197153586) (17 m, 129 passende Punkte) (https://commons.wikimedia.org/wiki/File:Goldauer_Bergsturz_(14197153586).jpg) | Bildsuche: CH.SZ.Arth.Goldau Rossberg Gnipen 2016-10-30 92 16x9-R 5120x2880 (219 passende Punkte) (https://commons.wikimedia.org/wiki/File:CH.SZ.Arth.Goldau_Rossberg_Gnipen_2016-10-30_92_16x9-R_5120x2880.jpg)</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2162,7 +2125,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>2026-10-23T23:21:39Z</t>
+          <t>2026-10-24T08:08:05Z</t>
         </is>
       </c>
     </row>
@@ -2192,12 +2155,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Pfarrkirche Herz-Jesu Goldau</t>
+          <t>Pfarrkirche Herz-Jesu</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Rossberg</t>
+          <t>Rigi Kulm; Rossberg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2211,38 +2174,38 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>47.0475</v>
+        <v>47.046563</v>
       </c>
       <c r="K17" t="n">
-        <v>8.5465</v>
+        <v>8.544949000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>2684183</v>
+        <v>2684067</v>
       </c>
       <c r="M17" t="n">
-        <v>1211313</v>
+        <v>1211207</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S17" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2257,7 +2220,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Verifiziertes Referenzfoto «Goldau von Südwesten» zeigt dieselbe Szene. (https://commons.wikimedia.org/wiki/File:Goldau_von_S%C3%BCdwesten.jpg) | Amtliches Adressverzeichnis: Gotthardstrasse 36 liegt in der Ortschaft Goldau (6410). | GWR führt die Pfarrkirche Goldau in der Ortschaft Goldau. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190166532_0)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die neuromanische Kirche mit Steinturm und Kupferhelm direkt an der Autobahn A4, dazu die Bahnanlagen und der Coop am Bahnhof, passen zur Herz-Jesu-Kirche in Goldau; das Bild ist vom Rossberg aus gegen den bewaldeten Rigihang aufgenommen.</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -2267,7 +2230,7 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>2026-10-23T23:21:46Z</t>
+          <t>2026-10-24T08:08:10Z</t>
         </is>
       </c>
     </row>
@@ -2297,12 +2260,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Talstation Stuckli Rondo (Sattel-Hochstuckli); Pfarrkirche St. Peter und Paul</t>
+          <t>Talstation Stuckli Rondo</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Kreisel</t>
+          <t>Kreisel 2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2311,38 +2274,38 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>47.0787</v>
+        <v>47.078433</v>
       </c>
       <c r="K18" t="n">
-        <v>8.635199999999999</v>
+        <v>8.634439</v>
       </c>
       <c r="L18" t="n">
-        <v>2690870</v>
+        <v>2690813</v>
       </c>
       <c r="M18" t="n">
-        <v>1214880</v>
+        <v>1214849</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="Q18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR), Bildinhalt); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR), Karte); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2362,7 +2325,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt der Parkplatz bei der Talstation (Kreisel 2/4) in der Ortschaft Sattel (PLZ 6417). | Das Session-Foto SG.CIV.17.144 wurde der Ortschaft Sattel zugeordnet; SG.CIV.17.177 zeigt die Hängebrücke am Hochstuckli. | Im GWR ist die Talstation Stuckli Rondo unter Kreisel 2 in der Ortschaft Sattel verzeichnet. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190194959_0)</t>
+          <t>Vergleichsfoto vor Ort: Mapillary Sattel 2017-04-22 (163 m, 181 passende Punkte) (https://www.mapillary.com/app/?pKey=1198343227335019) | Vergleichsfoto vor Ort: Mapillary Sattel 2017-04-22 (147 m, 169 passende Punkte) (https://www.mapillary.com/app/?pKey=398219548162763) | Bildsuche: Mapillary Sattel 2022-09-01 (101 passende Punkte) (https://www.mapillary.com/app/?pKey=559738142599040)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2372,7 +2335,7 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>2026-10-23T23:22:29Z</t>
+          <t>2026-10-24T08:08:15Z</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2365,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Chaiserstock; Blüemberg</t>
+          <t>Chaiserstock; Chronenstock; Glärnisch; Rossstock</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2411,38 +2374,38 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>46.9595</v>
+        <v>46.957436</v>
       </c>
       <c r="K19" t="n">
-        <v>8.657</v>
+        <v>8.674626</v>
       </c>
       <c r="L19" t="n">
-        <v>2692731</v>
+        <v>2694076</v>
       </c>
       <c r="M19" t="n">
-        <v>1201655</v>
+        <v>1201447</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, swisstopo-Ortsname); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, swisstopo-Ortsname); Gebäude, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2462,7 +2425,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Laut amtlichem Ortschaftenverzeichnis liegt der Kamerastandort auf dem Stooser Grat in der Ortschaft Stoos SZ (6433). | Ein verifiziertes Referenzfoto des Chaiserstocks (513 Inlier) wurde vom Grat zwischen Fronalpstock und Klingenstock aus aufgenommen. (https://commons.wikimedia.org/wiki/File:Chaiserstock.jpg) | Laut swisstopo liegt der Klingenstock am Stooser Grat in der Gemeinde Morschach, die Klingenstockbahn führt von Stoos dorthin. (https://api3.geo.admin.ch/rest/services/api/SearchServer?searchText=Klingenstock&amp;type=locations&amp;sr=2056&amp;limit=8)</t>
+          <t>2 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'web': Der spitze Felszahn mit dem breiten Felsklotz links davon passt zu Chaiserstock und Chronenstock über dem Riemenstaldnertal. Die Wanderer gehen auf einem grasigen Gratweg, vermutlich am Gratweg Klingenstock–Fronalpstock ob Stoos. | swissNAMES3D (swisstopo)</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -2472,7 +2435,7 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>2026-10-23T23:23:48Z</t>
+          <t>2026-10-24T08:08:31Z</t>
         </is>
       </c>
     </row>
@@ -2490,14 +2453,29 @@
       <c r="C20" t="n">
         <v>1</v>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Rigi Scheidegg</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Schwyz</t>
+          <t>Gersau</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Marienkapelle (Ibergeregg)</t>
+          <t>Kapelle Rigi Scheidegg</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Fronalpstock; Rigi Kulm; Vierwaldstättersee</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Rigi Scheidegg 92</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2506,43 +2484,38 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>47.0166</v>
+        <v>47.027263</v>
       </c>
       <c r="K20" t="n">
-        <v>8.7333</v>
+        <v>8.520979000000001</v>
       </c>
       <c r="L20" t="n">
-        <v>2698433</v>
+        <v>2682275</v>
       </c>
       <c r="M20" t="n">
-        <v>1208095</v>
+        <v>1209036</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0</v>
+        <v>0.571</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0</v>
+        <v>0.571</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0</v>
+        <v>0.571</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0</v>
+        <v>0.571</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Gemeinde durch eine Quelle gestützt (Gebäuderegister (OSM/GWR)); Ortschaft, See/Fluss/Berg, Strasse nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Schwyz / nicht bestimmbar); Prüfung nötig.</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Ortschaft, See/Fluss/Berg, Strasse</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr">
@@ -2557,7 +2530,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>OpenStreetMap verortet die Marienkapelle am Ibergeregg in der Gemeinde Schwyz. (https://www.openstreetmap.org/way/247989959) | OpenStreetMap führt die Marienkapelle am Ibergeregg-Pass als Kapelle in Passlage mit Fernsicht, was zur abgebildeten Holzkapelle passt. (https://www.openstreetmap.org/way/247989959) | Kleine Holzschindelkapelle mit schwarzem Spitzhelm und Kreuzigungsgruppe am Giebel auf einer Geländekante mit Blick auf verschneite Alpen.</t>
+          <t>Vergleichsfoto vor Ort: 1646-Rigi-Scheidegg (28 m, 79 passende Punkte) (https://commons.wikimedia.org/wiki/File:1646-Rigi-Scheidegg.jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 1 von 3 unabhängigen Untersuchungen nennen diese Gemeinde</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -2567,7 +2540,7 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>2026-10-23T23:24:20Z</t>
+          <t>2026-10-24T08:08:47Z</t>
         </is>
       </c>
     </row>
@@ -2597,17 +2570,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Stall Graussli (Sommerschwendistrasse 19); Wohnhaus Sommerschwendistrasse 20</t>
+          <t>Stall Graussli / Gebäude-Nr. 33</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Rigi Hochflue; Rigi</t>
+          <t>Rigiaa; Brunnen-Urmiberg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Sommerschwendistrasse 20</t>
+          <t>Sommerschwendistrasse 19</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2616,38 +2589,38 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>47.0774</v>
+        <v>47.077391</v>
       </c>
       <c r="K21" t="n">
-        <v>8.6355</v>
+        <v>8.63522</v>
       </c>
       <c r="L21" t="n">
-        <v>2690895</v>
+        <v>2690874</v>
       </c>
       <c r="M21" t="n">
-        <v>1214736</v>
+        <v>1214734</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR)). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2662,7 +2635,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet den Punkt der Ortschaft Sattel (PLZ 6417) zu. | Das Session-Foto zeigt die Talstation Stuckli Rondo in Sattel, von der aus die Gondel über diesen Hof fährt. | Im GWR liegt der Stall Graussli an der Sommerschwendistrasse 19 in der Ortschaft Sattel. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/191586373_0)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'web': Das Bild aus derselben Serie zeigt die Hängebrücke Skywalk von Sattel-Hochstuckli. Diese Aufnahme ist schräg von oben aus der Gondel kurz nach der Talstation in Sattel gemacht, Blick nach Südwesten Richtung Hochflue. Unten sieht man Wohnhaus und alten Stall an der Sommerschwendistrasse (Graussli), direkt unter der Bahnlinie.</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -2672,7 +2645,7 @@
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>2026-10-23T23:25:09Z</t>
+          <t>2026-10-24T08:08:28Z</t>
         </is>
       </c>
     </row>
@@ -2692,17 +2665,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Brunnen</t>
+          <t>Lauerz</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ingenbohl</t>
+          <t>Lauerz</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Rigi Hochflue; Urmiberg</t>
+          <t>Rossberg</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2711,38 +2684,38 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>46.999</v>
+        <v>47.02795028686523</v>
       </c>
       <c r="K22" t="n">
-        <v>8.574999999999999</v>
+        <v>8.586529731750488</v>
       </c>
       <c r="L22" t="n">
-        <v>2686427</v>
+        <v>2687257</v>
       </c>
       <c r="M22" t="n">
-        <v>1205952</v>
+        <v>1209183</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.6</v>
+        <v>0.571</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Geländeprüfung); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Bildinhalt); Gebäude, Strasse nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Brunnen, Ingenbohl / Gersau); Prüfung nötig.</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2762,7 +2735,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Das amtliche Ortschaftenverzeichnis ordnet den vermuteten Standort südlich der Hochflue der Ortschaft Brunnen (6440) zu. | Die Skyline-Berechnung von Ingenbohl-Wylen ergibt für den Grat Hochflue–Gottertli–Stockflue Höhenwinkel von 17–21°, passend zum Bild. | Laut swissBOUNDARIES3D liegt der vermutete Standort in der Gemeinde Ingenbohl.</t>
+          <t>3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Altes Blockhaus mit Bruchsteinsockel unter einer Kalkfelswand mit bewaldetem Grat, die nach rechts abfällt, dazu viele Hochspannungsleitungen. Das passt vermutlich zur Hochflue-Nordseite bei Lauerz; Schrift gibt es keine, darum nur eine Vermutung. | Untersuchung 'web': Altes Blockhaus auf Bruchsteinsockel; dahinter eine Kalkfelswand mit bewaldetem Hang und Hochspannungsleitungen, die an die Südseite der Rigi Hochflue über Lauerz erinnert. Kein Text lesbar, Zuordnung nur vermutet.</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -2772,7 +2745,7 @@
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>2026-10-23T23:25:20Z</t>
+          <t>2026-10-24T08:08:16Z</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2775,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Kehrichtverbrennungsanlage (Ringstrasse 81); Talstation LSBF</t>
+          <t>Stoos-Seeli Steg</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2810,54 +2783,54 @@
           <t>Stoos-Seeli</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Ringstrasse 81</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>08.10.2010</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>46.9755</v>
+        <v>46.97519</v>
       </c>
       <c r="K23" t="n">
-        <v>8.661899999999999</v>
+        <v>8.661735999999999</v>
       </c>
       <c r="L23" t="n">
-        <v>2693076</v>
+        <v>2693064</v>
       </c>
       <c r="M23" t="n">
-        <v>1203439</v>
+        <v>1203405</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.95</v>
+        <v>0.571</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="S23" s="3" t="n">
-        <v>0.9</v>
+        <v>0.571</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Karte, Gebäuderegister (OSM/GWR), Bildinhalt); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte). In 2 unabhängigen Analysen übereinstimmend.</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>nein</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Strasse</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -2867,7 +2840,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Das amtliche Ortschaftenverzeichnis ordnet den Stoos-Seeli und die Ringstrasse 81 der Ortschaft Stoos SZ (6433) zu. | Das Luftbild 2010 zeigt Seeform, Weg und Dorfanlage genau wie auf dem Foto. | Das GWR führt die Gebäude am See unter der Ortschaft Stoos SZ. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190102722_0)</t>
+          <t>3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'web': Blick von oben (Hang des Fronalpstocks) auf den 2008/09 gebauten Speichersee Stoos-Seeli mit Ringweg und dem autofreien Chaletdorf Stoos daneben; Lage und Form des Sees passen zum Registerpunkt. | swissNAMES3D (swisstopo)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2877,7 +2850,7 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-10-23T23:27:01Z</t>
+          <t>2026-10-24T08:08:18Z</t>
         </is>
       </c>
     </row>
@@ -2905,14 +2878,9 @@
           <t>Schwyz</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>ehemaliges Postgebäude Ibach</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Gotthardstrasse 69</t>
+          <t>Schmiedgasse 94</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2921,43 +2889,43 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>47.01103</v>
+        <v>47.01392</v>
       </c>
       <c r="K24" t="n">
-        <v>8.643890000000001</v>
+        <v>8.645593999999999</v>
       </c>
       <c r="L24" t="n">
-        <v>2691645</v>
+        <v>2691770</v>
       </c>
       <c r="M24" t="n">
-        <v>1207368</v>
+        <v>1207691</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Session-Foto); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Session-Foto); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>See/Fluss/Berg</t>
+          <t>Gebäude, See/Fluss/Berg</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -2972,7 +2940,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Verifizierte Archivkarte «Vordere Muotabrücke, Ibach» (1907, Aufschrift «Postgebäude in Ibach») zeigt dasselbe Haus mit Eckturm. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=357395) | Amtliches Adressverzeichnis: Gotthardstrasse 69 liegt in der Ortschaft 6438 Ibach. | Session-Fotos zeigen den Talkessel Schwyz, zu dem Ibach gehört.</t>
+          <t>Bildsuche: Mapillary Schwyz 2020-05-08 (272 passende Punkte) (https://www.mapillary.com/app/?pKey=1057456008398636) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -2982,7 +2950,7 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>2026-10-23T23:27:32Z</t>
+          <t>2026-10-24T08:09:03Z</t>
         </is>
       </c>
     </row>
@@ -3012,12 +2980,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Kantonsschule Kollegium Schwyz; Staatsarchiv des Kantons Schwyz</t>
+          <t>Kantonsschule Kollegium Schwyz</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Kollegiumstrasse 28</t>
+          <t>Kollegiumstrasse 30</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3026,38 +2994,38 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>47.02435</v>
+        <v>47.024435</v>
       </c>
       <c r="K25" t="n">
-        <v>8.653499999999999</v>
+        <v>8.653551</v>
       </c>
       <c r="L25" t="n">
-        <v>2692353</v>
+        <v>2692357</v>
       </c>
       <c r="M25" t="n">
-        <v>1208860</v>
+        <v>1208869</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="Q25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S25" s="3" t="n">
-        <v>1</v>
+        <v>0.962</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Gebäuderegister (OSM/GWR), Bildinhalt); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Gebäuderegister (OSM/GWR), Session-Foto); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3077,7 +3045,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis von swisstopo liegt das Kollegium in der Ortschaft Schwyz (PLZ 6430). | Ein bestätigtes Vergleichsfoto von 2013 zeigt die Kantonsschule Kollegium Schwyz in Schwyz. (https://commons.wikimedia.org/wiki/File:Schwyz_-_panoramio_(30).jpg) | In OpenStreetMap steht die Kantonsschule Kollegium Schwyz in der Gemeinde Schwyz. (https://www.openstreetmap.org/way/239379560)</t>
+          <t>Vergleichsfoto vor Ort: Schwyz - panoramio (14) (162 m, 84 passende Punkte) (https://commons.wikimedia.org/wiki/File:Schwyz_-_panoramio_(14).jpg) | Bildsuche: Schwyz - panoramio (30) (452 passende Punkte) (https://commons.wikimedia.org/wiki/File:Schwyz_-_panoramio_(30).jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -3087,7 +3055,7 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>2026-10-23T23:30:07Z</t>
+          <t>2026-10-24T08:08:53Z</t>
         </is>
       </c>
     </row>
@@ -3107,22 +3075,27 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Alpthal</t>
+          <t>Unteriberg</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Alpthal</t>
+          <t>Schwyz</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Br. Klausenkapelle Holzegg</t>
+          <t>Laucherenchappelen</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Spirstock</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Holzegg 1.7</t>
+          <t>Spirstock 1.2</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3131,48 +3104,43 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>47.028898</v>
+        <v>47.003326</v>
       </c>
       <c r="K26" t="n">
-        <v>8.700132999999999</v>
+        <v>8.767246999999999</v>
       </c>
       <c r="L26" t="n">
-        <v>2695890</v>
+        <v>2701039</v>
       </c>
       <c r="M26" t="n">
-        <v>1209421</v>
+        <v>1206663</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>0.5</v>
+        <v>0.923</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>0.75</v>
+        <v>0.923</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>See/Fluss/Berg</t>
-        </is>
-      </c>
-      <c r="V26" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -3182,7 +3150,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt die Kapelle (Holzegg 1.7) in der Ortschaft Alpthal, PLZ 8849. | OSM führt die Br. Klausenkapelle Holzegg in Alpthal. (https://www.openstreetmap.org/way/198077020) | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Alpthal).</t>
+          <t>Vergleichsfoto vor Ort: Hoch-Ybrig - panoramio (107) (120 m, 177 passende Punkte) (https://commons.wikimedia.org/wiki/File:Hoch-Ybrig_-_panoramio_(107).jpg) | Bildsuche: Hoch-Ybrig - panoramio (107) (177 passende Punkte) (https://commons.wikimedia.org/wiki/File:Hoch-Ybrig_-_panoramio_(107).jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -3192,7 +3160,7 @@
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>2026-10-23T23:29:03Z</t>
+          <t>2026-10-24T08:09:27Z</t>
         </is>
       </c>
     </row>
@@ -3248,26 +3216,26 @@
         <v>1217844</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="Q27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S27" s="3" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Text im Bild, Gebäudeadressverzeichnis, Referenzfoto); Gemeinde durch 4 unabhängige Quellen gestützt (Text im Bild, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Referenzfoto); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3287,7 +3255,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Die Anschlagtafel im Vordergrund trägt die Aufschrift «Gemeinde Rothenthurm – Amtliche Anzeigen». | Laut swisstopo liegen die Kirchenkoordinaten in der Ortschaft Rothenthurm (6418). | Ein bestätigter Treffer zeigt die Pfarrkirche Rothenthurm. (https://commons.wikimedia.org/wiki/File:Rothenthurm_Pfarrkirche.jpg)</t>
+          <t>Bildsuche: Rothenthurm Pfarrkirche (616 passende Punkte) (https://commons.wikimedia.org/wiki/File:Rothenthurm_Pfarrkirche.jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
@@ -3297,7 +3265,7 @@
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>2026-10-23T23:28:30Z</t>
+          <t>2026-10-24T08:09:11Z</t>
         </is>
       </c>
     </row>
@@ -3353,26 +3321,26 @@
         <v>1220262</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S28" s="3" t="n">
-        <v>0.6</v>
+        <v>0.962</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Einsiedeln / nicht bestimmbar); Prüfung nötig.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3380,9 +3348,9 @@
           <t>See/Fluss/Berg</t>
         </is>
       </c>
-      <c r="V28" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
@@ -3392,7 +3360,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Die amtliche Adresssuche an der Reithalle ergibt die Ortschaft Einsiedeln (8840). | OSM verzeichnet an dieser Stelle die Reithalle Reitverein Einsiedeln. (https://www.openstreetmap.org/way/192914714) | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Einsiedeln).</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Moderne Holz-Reithalle mit Stalltrakt, Plakette «Equigarde 2004» (Pferdestall-Label) und Infotafel mit Pferdelogo «Marstall … Einsiedeln»; passt zur Reithalle beim Marstall des Klosters Einsiedeln.</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -3402,7 +3370,7 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>2026-10-23T23:30:00Z</t>
+          <t>2026-10-24T08:09:15Z</t>
         </is>
       </c>
     </row>
@@ -3432,17 +3400,17 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>McDonald's Seewen; Gewerbehalle Bahnhofstrasse 192</t>
+          <t>Riedmattli</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Kleiner Mythen; Grosser Mythen</t>
+          <t>Gross Mythen; Chli Mythen</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Bahnhofstrasse</t>
+          <t>Riedmattli 3</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3451,38 +3419,38 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>47.03085</v>
+        <v>47.030574</v>
       </c>
       <c r="K29" t="n">
-        <v>8.62649</v>
+        <v>8.626182999999999</v>
       </c>
       <c r="L29" t="n">
-        <v>2690289</v>
+        <v>2690266</v>
       </c>
       <c r="M29" t="n">
-        <v>1209551</v>
+        <v>1209520</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>0.5</v>
+        <v>0.923</v>
       </c>
       <c r="S29" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -3497,7 +3465,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Die amtliche Adressabfrage am Kreisel ergibt Ortschaft Seewen SZ (PLZ 6423). | Das im Bild sichtbare McDonald's liegt laut OSM an der Steinbislin 5 in Seewen, Gemeinde Schwyz. (https://www.openstreetmap.org/way/31859285) | Die Standortberechnung aus Kleinem und Grossem Mythen ergibt Kamerastandorte in Seewen SZ mit Blick nach Nordosten.</t>
+          <t>Vergleichsfoto vor Ort: Mapillary Schwyz 2025-06-14 (67 m, 125 passende Punkte) (https://www.mapillary.com/app/?pKey=613436188453471) | Vergleichsfoto vor Ort: Mapillary Schwyz 2021-10-19 (73 m, 113 passende Punkte) (https://www.mapillary.com/app/?pKey=4287978487997718) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3507,7 +3475,7 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>2026-10-23T23:31:55Z</t>
+          <t>2026-10-24T08:09:29Z</t>
         </is>
       </c>
     </row>
@@ -3542,7 +3510,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Rigi Hochflue; Urmiberg; Vierwaldstättersee</t>
+          <t>Brunnen-Urmiberg; Vierwaldstättersee</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3556,10 +3524,10 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>46.9771</v>
+        <v>46.977101</v>
       </c>
       <c r="K30" t="n">
-        <v>8.6145</v>
+        <v>8.614497999999999</v>
       </c>
       <c r="L30" t="n">
         <v>2689467</v>
@@ -3568,26 +3536,26 @@
         <v>1203562</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S30" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -3602,7 +3570,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Laut amtlichem Ortschaftenverzeichnis liegt das Antoniushaus Mattli in der Ortschaft Morschach (PLZ 6443). | OSM führt das Antoniushaus Mattli in der Gemeinde Morschach. (https://www.openstreetmap.org/way/184735124) | Die berechnete Skyline von südöstlich des Mattli (Rigi Hochflue, Gottertli) und der Sonnenstand passen zum Bild.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die gestaffelte Anlage aus Sichtbeton mit Holz-Fensterelementen (Béton brut, Adelbert Koch 1965–67) auf der Geländeterrasse über Brunnen und dem See ist das Mattli Antoniushaus in Morschach.</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -3612,7 +3580,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>2026-10-23T23:34:32Z</t>
+          <t>2026-10-24T08:09:16Z</t>
         </is>
       </c>
     </row>
@@ -3632,22 +3600,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Morschach</t>
+          <t>Vorderthal</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Morschach</t>
+          <t>Vorderthal</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Pfarrkirche Morschach</t>
+          <t>Pfarrkirche Peter und Paul</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Schiltistrasse 3a</t>
+          <t>Wägitalstrasse 49a.1</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3656,38 +3624,38 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>46.9817</v>
+        <v>47.122687</v>
       </c>
       <c r="K31" t="n">
-        <v>8.6195</v>
+        <v>8.899328000000001</v>
       </c>
       <c r="L31" t="n">
-        <v>2689840</v>
+        <v>2710835</v>
       </c>
       <c r="M31" t="n">
-        <v>1204079</v>
+        <v>1220109</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S31" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3707,7 +3675,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Verifiziertes Referenzfoto (59 Inlier) zeigt dieselbe Dorfansicht von Morschach. (https://commons.wikimedia.org/wiki/File:Lake_Luzern_(Lucerne)_Area,_Morschach_Village_(9808406374).jpg) | Das amtliche Adressverzeichnis ordnet die Pfarrkirche der Ortschaft 6443 Morschach zu. | Im GWR ist die Pfarrkirche Morschach mit der Ortschaft Morschach eingetragen. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190287408_0)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 2 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Bergdorf in engem Tal mit steilen Wald- und Wiesenhängen, kleine barocke Kirche mit Spitzhelm und Uhr, daneben eine Gruppe neuer Mehrfamilienhäuser (passt zur Überbauung Postwiese westlich der Kirche Vorderthal). Lesbaren Text gibt es keinen; die Zuordnung zum Wägital ist eine Vermutung.</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3717,7 +3685,7 @@
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>2026-10-23T23:32:20Z</t>
+          <t>2026-10-24T08:10:36Z</t>
         </is>
       </c>
     </row>
@@ -3747,12 +3715,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Pfarrkirche St. Gallus; Swiss Holiday Park</t>
+          <t>Pfarrhaus</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Dorfstrasse</t>
+          <t>Schiltistrasse 1</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3761,38 +3729,38 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>46.98172</v>
+        <v>46.981495</v>
       </c>
       <c r="K32" t="n">
-        <v>8.618499999999999</v>
+        <v>8.618931999999999</v>
       </c>
       <c r="L32" t="n">
-        <v>2689764</v>
+        <v>2689797</v>
       </c>
       <c r="M32" t="n">
-        <v>1204080</v>
+        <v>1204056</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S32" s="3" t="n">
-        <v>1</v>
+        <v>0.962</v>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Text im Bild, Referenzfoto, Gebäudeadressverzeichnis, Session-Foto); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Text im Bild, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3812,7 +3780,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Auf der Sitzbank steht 'Morschach Tourismus'. | Ein verifiziertes Referenzfoto 'House in Morschach' zeigt dasselbe Holzhaus. (https://commons.wikimedia.org/wiki/File:Lake_Luzern_(Lucerne)_Area,_House_in_Morschach_(9808475583).jpg) | Laut amtlichem Ortschaftenverzeichnis liegt der Punkt an der Dorfstrasse in der Ortschaft 6443 Morschach.</t>
+          <t>Bildsuche: Lake Luzern (Lucerne) Area, House in Morschach (9808475583) (141 passende Punkte) (https://commons.wikimedia.org/wiki/File:Lake_Luzern_(Lucerne)_Area,_House_in_Morschach_(9808475583).jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
@@ -3822,7 +3790,7 @@
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>2026-10-23T23:33:34Z</t>
+          <t>2026-10-24T08:09:38Z</t>
         </is>
       </c>
     </row>
@@ -3869,35 +3837,35 @@
         <v>46.981932</v>
       </c>
       <c r="K33" t="n">
-        <v>8.619856</v>
+        <v>8.619846000000001</v>
       </c>
       <c r="L33" t="n">
-        <v>2689867</v>
+        <v>2689866</v>
       </c>
       <c r="M33" t="n">
         <v>1204105</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q33" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S33" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto, Text im Bild); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3917,7 +3885,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt Dorfstrasse 22 in der Ortschaft 6443 Morschach. | Das GWR führt das Hotel Betschart an der Dorfstrasse 22 in der Ortschaft Morschach. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190211680_0) | Ein Foto derselben Aufnahmeserie zeigt das Pfarrhaus Morschach im Dorfzentrum.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Schriftzug «BETSCHART» und Pizzeria «Roma» am Gebäude passen zum Hotel Betschart an der Dorfstrasse 22 in Morschach; die Fotos derselben Serie zeigen Morschacher Dorfansichten mit dem Swiss-Holiday-Park-Bau.</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -3927,7 +3895,7 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>2026-10-23T23:34:28Z</t>
+          <t>2026-10-24T08:09:56Z</t>
         </is>
       </c>
     </row>
@@ -3947,27 +3915,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Morschach</t>
+          <t>Seewen SZ</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Morschach</t>
+          <t>Schwyz</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Pfarrkirche St. Gallus</t>
+          <t>Kirche</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Kleiner Mythen; Grosser Mythen</t>
+          <t>Gross Mythen; Chli Mythen; Rigi</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Schiltistrasse 3a</t>
+          <t>Engibergweg 2</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3976,38 +3944,38 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>46.98155</v>
+        <v>47.029707</v>
       </c>
       <c r="K34" t="n">
-        <v>8.620050000000001</v>
+        <v>8.630808999999999</v>
       </c>
       <c r="L34" t="n">
-        <v>2689882</v>
+        <v>2690619</v>
       </c>
       <c r="M34" t="n">
-        <v>1204063</v>
+        <v>1209429</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>0.95</v>
+        <v>0.571</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.95</v>
+        <v>0.571</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="S34" s="3" t="n">
-        <v>0.6</v>
+        <v>0.571</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäuderegister (OSM/GWR), Geländeprüfung, Session-Foto, Gebäudeadressverzeichnis); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäuderegister (OSM/GWR), Karte, Session-Foto, Gebäudeadressverzeichnis). Zwei unabhängige Analysen nennen verschiedene Orte (Morschach / Schwyz); Prüfung nötig.</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V34" s="4" t="inlineStr">
@@ -4022,7 +3990,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Das GWR führt die Pfarrkirche Morschach an der Schiltistrasse 3a in der Ortschaft Morschach. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190287408_0) | Die Standortberechnung aus Kleinem und Grossem Mythen (130 mm Brennweite) ergibt eine Kurve auf der Breite der Morschacher Terrasse, Blick nach Nordosten. | Das Session-Foto zeigt das Erlebnisbad mit Rutsche und einen Skilift (Swiss Holiday Park Morschach).</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 1 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die beiden Mythen von Westen gesehen, davor eine alte Kirche mit Dachreiter am Fuss des felsigen, bewaldeten Engibergs; das passt zur Alten Kapelle Seewen am Engibergweg 2. Die Fotos aus derselben Serie mit der Terrassensiedlung und dem Parkplatz sprechen für den Ortskern von Seewen.</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -4032,7 +4000,7 @@
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>2026-10-23T23:35:20Z</t>
+          <t>2026-10-24T08:10:56Z</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4030,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Pfarrhaus Morschach; Hotel Axenfels (Swiss Holiday Park)</t>
+          <t>Pfarrhaus</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4088,26 +4056,26 @@
         <v>1204056</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4127,7 +4095,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Das amtliche Adressregister ordnet den Punkt des Pfarrhauses der Ortschaft Morschach (PLZ 6443) zu. | Das Session-Foto zeigt das Hotel Betschart an der Dorfstrasse 22 in Morschach. | Laut OSM steht das Pfarrhaus an der Schiltistrasse 1 in Morschach, neben dem Swiss Holiday Park. (https://www.openstreetmap.org/way/199605454)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Im Hintergrund steht der weiss-rote Hotelbau des Swiss Holiday Park in Morschach. Davor ist ein Blockbau mit steilem Giebel, Klebdächern und Sichtfachwerk im hinteren Teil zu sehen. Das passt zur Beschreibung des Pfarrhauses von 1685 an der Schiltistrasse 1, das direkt neben dem Holiday Park steht.</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -4137,7 +4105,7 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>2026-10-23T23:37:10Z</t>
+          <t>2026-10-24T08:09:50Z</t>
         </is>
       </c>
     </row>
@@ -4167,17 +4135,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Kloster St. Josef; Primarschule St. Josef</t>
+          <t>Frauenkloster St. Josef</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Muota</t>
+          <t>Muotatal</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Kloster St. Josef 1</t>
+          <t>Kloster St. Josef 1 - 2</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4186,38 +4154,38 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>46.97575</v>
+        <v>46.975794</v>
       </c>
       <c r="K36" t="n">
-        <v>8.763450000000001</v>
+        <v>8.763347</v>
       </c>
       <c r="L36" t="n">
-        <v>2700802</v>
+        <v>2700794</v>
       </c>
       <c r="M36" t="n">
-        <v>1203593</v>
+        <v>1203597</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S36" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -4232,7 +4200,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet den Klosterstandort der Ortschaft Muotathal (6436) zu. | OSM führt das Kloster St. Josef in Muotathal. (https://www.openstreetmap.org/way/786971733) | Das Luftbild 2005 zeigt dieselbe Anlage mit Klosterhof, Scheune, Schulhaus und der Muota.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Typische Klosteranlage mit rotem Dachreiter, Klostermauer, Garten und grosser Scheune an der Muota – das Frauenkloster St. Josef in Muotathal, vom Hang oberhalb aus aufgenommen.</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -4242,7 +4210,7 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>2026-10-23T23:35:23Z</t>
+          <t>2026-10-24T08:10:02Z</t>
         </is>
       </c>
     </row>
@@ -4272,12 +4240,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Restaurant Grosser Mythen (Gipfelhütte)</t>
+          <t>Restaurant Grosser Mythen</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Grosser Mythen; Fronalpstock; Urner Alpen</t>
+          <t>Fronalpstock; Gross Mythen</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4291,38 +4259,38 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>47.02972</v>
+        <v>47.029702</v>
       </c>
       <c r="K37" t="n">
-        <v>8.68885</v>
+        <v>8.688834999999999</v>
       </c>
       <c r="L37" t="n">
-        <v>2695031</v>
+        <v>2695030</v>
       </c>
       <c r="M37" t="n">
-        <v>1209499</v>
+        <v>1209497</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>0.85</v>
+        <v>0.923</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>0.5</v>
+        <v>0.923</v>
       </c>
       <c r="S37" s="3" t="n">
-        <v>0.9</v>
+        <v>0.923</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Referenzfoto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -4337,7 +4305,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet den Gipfel des Grossen Mythen der Ortschaft 6430 Schwyz zu (Mythen 1). | Verifiziertes Referenzbild 'Gipfelhütte auf dem Großen Mythen' zeigt dieselbe Hütte. (https://commons.wikimedia.org/wiki/File:Gipfelh%C3%BCtte_auf_dem_Gro%C3%9Fen_Mythen.jpg) | Verifizierte Archivkarte 'Mythengebiet mit seinen Bergen' zeigt dieselbe Gipfelhütte. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=868591)</t>
+          <t>Vergleichsfoto vor Ort: 1893-Mythen-SW (24 m, 134 passende Punkte) (https://commons.wikimedia.org/wiki/File:1893-Mythen-SW.jpg) | Vergleichsfoto vor Ort: Gipfelhütte auf dem Großen Mythen (17 m, 78 passende Punkte) (https://commons.wikimedia.org/wiki/File:Gipfelh%C3%BCtte_auf_dem_Gro%C3%9Fen_Mythen.jpg) | Amtliches Register (GWR, OSM, KGS) am Ort des Motivs</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -4347,7 +4315,7 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>2026-10-23T23:35:33Z</t>
+          <t>2026-10-24T08:10:20Z</t>
         </is>
       </c>
     </row>
@@ -4365,35 +4333,13 @@
       <c r="C38" t="n">
         <v>1</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Näfels</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Obersee (GL); Brünnelistock</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>03.05.2007</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>47.0865</v>
-      </c>
-      <c r="K38" t="n">
-        <v>9.012</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2719464</v>
-      </c>
-      <c r="M38" t="n">
-        <v>1216252</v>
-      </c>
       <c r="N38" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>0</v>
@@ -4402,7 +4348,7 @@
         <v>0</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>0</v>
@@ -4412,12 +4358,12 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis); Gemeinde, Gebäude, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Nicht im Kanton Schwyz: vermutlich Glarus Nord GL. Felder offen gelassen.</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Gemeinde, Gebäude, Strasse</t>
+          <t>Ortschaft, Gemeinde, Gebäude, See/Fluss/Berg, Strasse</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -4430,11 +4376,6 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>Verifizierte Ansichtskarte 'Obersee mit Brünnelistock' (1944) zeigt dieselbe Szene am Obersee bei Näfels. (http://doi.org/10.3932/ethz-a-000999066) | Amtliches Ortschaftenverzeichnis: Standort am Obersee liegt in der Ortschaft Näfels (8752). | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Näfels).</t>
-        </is>
-      </c>
       <c r="Y38" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4442,7 +4383,7 @@
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>2026-10-23T23:36:58Z</t>
+          <t>2026-10-24T08:10:03Z</t>
         </is>
       </c>
     </row>
@@ -4470,14 +4411,19 @@
           <t>Schwyz</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>BSZ Stiftung Seewen</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Grosser Mythen; Kleiner Mythen</t>
+          <t>Chli Mythen; Gross Mythen; Haggenspitzli; Rotenflue</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Bättigmatt</t>
+          <t>Hausmatt 9</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4486,48 +4432,43 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>47.0277</v>
+        <v>47.02748</v>
       </c>
       <c r="K39" t="n">
-        <v>8.630100000000001</v>
+        <v>8.632650999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>2690569</v>
+        <v>2690763</v>
       </c>
       <c r="M39" t="n">
-        <v>1209205</v>
+        <v>1209183</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>0</v>
+        <v>0.962</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>0.5</v>
+        <v>0.962</v>
       </c>
       <c r="S39" s="3" t="n">
-        <v>0.6</v>
+        <v>0.962</v>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Geländeprüfung); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Bildinhalt, Geländeprüfung); Gebäude nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Seewen SZ, Schwyz / Schwyz); Prüfung nötig.</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>Gebäude</t>
-        </is>
-      </c>
-      <c r="V39" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
@@ -4537,7 +4478,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>Die amtliche Adressabfrage beim vermuteten Standort der Überbauung ergibt die Ortschaft Seewen SZ (PLZ 6423). | Die Standortsuche anhand von Chli Mythen und Grossem Mythen ergibt eine Standortkurve durch Seewen. | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Seewen SZ).</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'web': Kleiner und Grosser Mythen von Westen gesehen, mit etwa 16° Abstand zwischen den Gipfeln. Das passt zu einem Standort in Seewen, etwa 4 km entfernt. Der moderne Gebäudekomplex mit verglastem Verbindungsbau dürfte die BSZ Stiftung an der Hausmatt sein, was aber nicht direkt bestätigt ist.</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -4547,7 +4488,7 @@
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>2026-10-23T23:38:12Z</t>
+          <t>2026-10-24T08:10:24Z</t>
         </is>
       </c>
     </row>
@@ -4590,7 +4531,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Ortschaft, Gemeinde, Gebäude, See/Fluss/Berg, Strasse nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Nicht im Kanton Schwyz: vermutlich Reichenbach im Kandertal BE. Felder offen gelassen.</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4608,11 +4549,6 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>Hartbelagpiste parallel zu doppelspuriger Bahnlinie und Hauptstrasse in hügeligem Voralpental – ein solcher Flugplatz existiert im Kanton Schwyz nicht. | Laut OSM/GWR gibt es im Kanton Schwyz nur den Flugplatz Wangen-Lachen sowie Modellflugplätze. (https://www.openstreetmap.org/node/6373761732)</t>
-        </is>
-      </c>
       <c r="Y40" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4620,7 +4556,7 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>2026-10-23T23:38:53Z</t>
+          <t>2026-10-24T08:10:22Z</t>
         </is>
       </c>
     </row>
@@ -4650,17 +4586,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Hotel Sonne (Rigi Klösterli)</t>
+          <t>Riedboden</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Rigi</t>
+          <t>Rigi Kulm</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Klösterliweg 12</t>
+          <t>Staffelweg 6</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4669,38 +4605,38 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>47.044043</v>
+        <v>47.04646</v>
       </c>
       <c r="K41" t="n">
-        <v>8.484513</v>
+        <v>8.485541</v>
       </c>
       <c r="L41" t="n">
-        <v>2679479</v>
+        <v>2679553</v>
       </c>
       <c r="M41" t="n">
-        <v>1210864</v>
+        <v>1211133</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S41" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Session-Foto, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
@@ -4715,7 +4651,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt Klösterliweg 12 in der Ortschaft Rigi Klösterli (PLZ 6410). | Auf dem Session-Foto SG.CIV.17.424 ist die Hotelaufschrift „Klösterli … Hirschen“ zu lesen. | Das GWR führt das Gebäude „Sonne“ unter der Ortschaft Rigi Klösterli. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/256462_0)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Auf einem anderen Bild derselben Serie steht «Klösterli Hirschen», also wurde in Rigi Klösterli fotografiert. Das erhöht stehende Belle-Epoque-Haus mit dem Jugendstil-Türmli (Anbau von 1899) ist das ehemalige Hotel Des Alpes, früher Pension Riedboden, am Staffelweg 6.</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4725,7 +4661,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>2026-10-23T23:39:16Z</t>
+          <t>2026-10-24T08:10:24Z</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4691,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Hochhaus Schiller A</t>
+          <t>Cafe Schiller</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Hochflue</t>
+          <t>Brunnen-Urmiberg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4774,38 +4710,38 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>47.001335</v>
+        <v>47.001293</v>
       </c>
       <c r="K42" t="n">
-        <v>8.588782999999999</v>
+        <v>8.588649999999999</v>
       </c>
       <c r="L42" t="n">
-        <v>2687471</v>
+        <v>2687461</v>
       </c>
       <c r="M42" t="n">
-        <v>1206227</v>
+        <v>1206222</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P42" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="R42" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="S42" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Session-Foto, Karte); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
@@ -4820,7 +4756,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>Laut amtlichem Adressverzeichnis liegt Gersauerstrasse 76 in der Ortschaft Brunnen (6440). | OSM führt das Hochhaus Schiller A an der Gersauerstrasse 76 in Ingenbohl/Brunnen. (https://www.openstreetmap.org/way/380536496) | Das Session-Foto zeigt den grossen Getreidesilo beim Bahnhof Brunnen, also dieselbe Gegend.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die Serie (Kornsilo Brunnen, Pfarrkirche Ingenbohl) verortet die Aufnahme in Brunnen; das markante Wohnhochhaus mit Restaurant im Erdgeschoss am Hangfuss ist das Hochhaus Schiller A (höchstes Wohnhaus im Kanton) an der Gersauerstrasse 76 mit Café Restaurant Schiller.</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -4830,7 +4766,7 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>2026-10-23T23:30:35Z</t>
+          <t>2026-10-24T08:10:49Z</t>
         </is>
       </c>
     </row>
@@ -4860,12 +4796,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Rathaus Schwyz; Hotel Wysses Rössli; Postgebäude Schwyz</t>
+          <t>Wysses Rössli</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Fronalpstock</t>
+          <t>Fronalpstock 1. Sektion</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4879,38 +4815,38 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>47.02095</v>
+        <v>47.020747</v>
       </c>
       <c r="K43" t="n">
-        <v>8.653449999999999</v>
+        <v>8.653472000000001</v>
       </c>
       <c r="L43" t="n">
-        <v>2692355</v>
+        <v>2692357</v>
       </c>
       <c r="M43" t="n">
-        <v>1208482</v>
+        <v>1208459</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P43" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="R43" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S43" s="3" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Text im Bild); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Referenzfoto, Bildinhalt). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
@@ -4925,7 +4861,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis von swisstopo ordnet Hauptplatz 3 der Ortschaft Schwyz (6430) zu. | Die verifizierte Staatsarchiv-Aufnahme «Rathaus Schwyz und Hotel Wysses Rössli, Hauptplatz» zeigt dieselbe Szene. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=357284) | Die verifizierte Commons-Aufnahme «Hauptplatz in Schwyz» zeigt denselben Platz. (https://commons.wikimedia.org/wiki/File:Hauptplatz_in_Schwyz.jpg)</t>
+          <t>Vergleichsfoto vor Ort: Rathaus Schwyz 11 (22 m, 285 passende Punkte) (https://commons.wikimedia.org/wiki/File:Rathaus_Schwyz_11.jpg) | Vergleichsfoto vor Ort: Mapillary Schwyz 2022-11-29 (25 m, 268 passende Punkte) (https://www.mapillary.com/app/?pKey=661237635794614) | Bildsuche: Schwyz - panoramio (5) (649 passende Punkte) (https://commons.wikimedia.org/wiki/File:Schwyz_-_panoramio_(5).jpg)</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
@@ -4935,7 +4871,7 @@
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>2026-10-23T23:39:01Z</t>
+          <t>2026-10-24T08:10:48Z</t>
         </is>
       </c>
     </row>
@@ -4965,12 +4901,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Café Haug (Postplatz 4); Haus Hauptplatz 5</t>
+          <t>Café Haug</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Postplatz</t>
+          <t>Postplatz 4</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4979,38 +4915,38 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>47.02078</v>
+        <v>47.020887</v>
       </c>
       <c r="K44" t="n">
-        <v>8.652900000000001</v>
+        <v>8.652639000000001</v>
       </c>
       <c r="L44" t="n">
-        <v>2692314</v>
+        <v>2692294</v>
       </c>
       <c r="M44" t="n">
-        <v>1208462</v>
+        <v>1208474</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="P44" s="3" t="n">
-        <v>0.95</v>
+        <v>0.923</v>
       </c>
       <c r="Q44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>0.7</v>
+        <v>0.923</v>
       </c>
       <c r="S44" s="3" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Text im Bild); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Referenzfoto, Archivdatensatz, Gebäuderegister (OSM/GWR)); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe A: Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5030,7 +4966,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet den Postplatz der Ortschaft Schwyz (6430) zu. | Verifizierter Treffer Herrengasse 5 in Schwyz zeigt dieselbe Bebauung. (https://commons.wikimedia.org/wiki/File:Herrengasse_5_in_Schwyz.jpg) | Verifizierter Treffer Haus Hirschen, Hirzengasse 9 in Schwyz. (https://commons.wikimedia.org/wiki/File:Schwyz_-_panoramio_(11).jpg)</t>
+          <t>Vergleichsfoto vor Ort: Mapillary Schwyz 2018-08-19 (84 m, 97 passende Punkte) (https://www.mapillary.com/app/?pKey=179051307443417) | Vergleichsfoto vor Ort: Mapillary Schwyz 2018-08-19 (41 m, 81 passende Punkte) (https://www.mapillary.com/app/?pKey=3925569524204408) | Bildsuche: Mapillary Schwyz 2020-05-08 (378 passende Punkte) (https://www.mapillary.com/app/?pKey=946924729407912)</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -5040,7 +4976,7 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>2026-10-23T23:42:54Z</t>
+          <t>2026-10-24T08:11:01Z</t>
         </is>
       </c>
     </row>
@@ -5060,17 +4996,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Schwyz</t>
+          <t>Brunnen</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Schwyz</t>
+          <t>Ingenbohl</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Unterschönenbuch (St. Wendelinkapelle)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Rigi Hochflue</t>
+          <t>Brunnen-Urmiberg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -5079,43 +5020,43 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>47.023</v>
+        <v>46.998631</v>
       </c>
       <c r="K45" t="n">
-        <v>8.651999999999999</v>
+        <v>8.630572000000001</v>
       </c>
       <c r="L45" t="n">
-        <v>2692242</v>
+        <v>2690654</v>
       </c>
       <c r="M45" t="n">
-        <v>1208708</v>
+        <v>1205974</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>0.7</v>
+        <v>0.571</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S45" s="3" t="n">
-        <v>0.6</v>
+        <v>0.571</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Geländeprüfung, Gebäudeadressverzeichnis, Text im Bild); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Geländeprüfung); Gebäude, Strasse nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Schwyz / Rickenbach b. Schwyz, Schwyz); Prüfung nötig.</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>Gebäude, Strasse</t>
+          <t>Strasse</t>
         </is>
       </c>
       <c r="V45" s="4" t="inlineStr">
@@ -5130,7 +5071,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>Die Standortsuche mit Rigi Hochflue und Grat ergibt Kamerastandorte im Ostteil von Schwyz mit Blick nach Westen. | Die Adressabfrage am besten Standort (Theodosiusweg/Oberfeld) liefert Ortschaft 6430 Schwyz. | Der Wegweiser 'Ibach' zeigt nach links, also liegt Ibach südlich des Standorts, was zu Schwyz mit Blick nach Westen passt.</t>
+          <t>3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'blind': Wegweiser «Ibach» mit Wander-/Velowegweisern, viele Hochspannungsleitungen (Unterwerk Ingenbohl) und der Blick nach Westen auf Rigi Hochflue mit dem nahen Urmiberg rechts sprechen für Unterschönenbuch (Ingenbohl); das genaue Haus ist geschätzt. | swissNAMES3D (swisstopo)</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
@@ -5140,7 +5081,7 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>2026-10-23T23:42:48Z</t>
+          <t>2026-10-24T08:10:55Z</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5111,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Hotel Axenfels; Swiss Holiday Park</t>
+          <t>Swiss Holiday Park</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Grosser Mythen; Kleiner Mythen</t>
+          <t>Gross Mythen; Chli Mythen</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Dorfstrasse 11</t>
+          <t>Dorfstrasse 10</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5189,38 +5130,38 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>46.981548</v>
+        <v>46.980955</v>
       </c>
       <c r="K46" t="n">
-        <v>8.617725999999999</v>
+        <v>8.618109</v>
       </c>
       <c r="L46" t="n">
-        <v>2689705</v>
+        <v>2689736</v>
       </c>
       <c r="M46" t="n">
-        <v>1204060</v>
+        <v>1203995</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P46" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S46" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)); Gemeinde durch 3 unabhängige Quellen gestützt (Referenzfoto, Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR)). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
@@ -5235,7 +5176,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>Verifiziertes Archivbild zeigt dasselbe Kur- und Sporthotel Axenfels in Morschach. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=606545) | Amtliches Adressverzeichnis ordnet Dorfstrasse 11 der Ortschaft Morschach (6443) zu. | GWR führt das Hotel Axenfels in der Ortschaft Morschach. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/3088311_0)</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Ein grosser weisser Hotelkomplex mit roten Fensterrahmen und Türmchen steht neben einem Badgebäude mit Glas-Tonnendach. Im Hintergrund sind Grosser und Kleiner Mythen von Süden zu sehen. Das passt zum Swiss Holiday Park in Morschach mit Hotel, Erlebnisbad und Asia-Restaurant.</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
@@ -5245,7 +5186,7 @@
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>2026-10-23T23:40:44Z</t>
+          <t>2026-10-24T08:10:59Z</t>
         </is>
       </c>
     </row>
@@ -5265,7 +5206,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Seewen SZ</t>
+          <t>Schwyz</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -5275,7 +5216,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Eidg. Zeughaus Seewen</t>
+          <t>Forum der Schweizergeschichte</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Zeughausstrasse 5</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5284,48 +5230,48 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>47.0262</v>
+        <v>47.021354</v>
       </c>
       <c r="K47" t="n">
-        <v>8.632999999999999</v>
+        <v>8.651616000000001</v>
       </c>
       <c r="L47" t="n">
-        <v>2690792</v>
+        <v>2692215</v>
       </c>
       <c r="M47" t="n">
-        <v>1209041</v>
+        <v>1208524</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="P47" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="Q47" s="3" t="n">
         <v>0</v>
       </c>
       <c r="R47" s="3" t="n">
-        <v>0</v>
+        <v>0.962</v>
       </c>
       <c r="S47" s="3" t="n">
-        <v>0.6</v>
+        <v>0.962</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>Ortschaft durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Archivdatensatz); Gemeinde durch 2 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Archivdatensatz); See/Fluss/Berg, Strasse nicht bestimmbar. Zwei unabhängige Analysen nennen verschiedene Orte (Seewen SZ, Schwyz / Schwyz); Prüfung nötig.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>See/Fluss/Berg, Strasse</t>
-        </is>
-      </c>
-      <c r="V47" s="4" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>See/Fluss/Berg</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>nein</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
@@ -5335,7 +5281,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>Das amtliche Ortschaftenverzeichnis ordnet das Gebiet beim Bahnhof Schwyz der Ortschaft Seewen SZ zu. | Die Archivkarte «Eidg. Zeughaus und Bahnhof in Seewen» (1916) belegt ein eidgenössisches Zeughaus direkt beim Bahnhof Seewen. (https://query.staatsarchiv.sz.ch/detail.aspx?ID=357205) | Automatische Prüfung: das amtliche Verzeichnis nennt am Antwortpunkt dieselbe Ortschaft (Seewen SZ).</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Langer Bruchsteinbau mit Remisentoren, Rundbogentüren und Signal «Werkverkehr» erinnert an einen historischen Militär-/Zeughausbau um 1900; vermutet wird das Zeughausareal Seewen (Schwyz). Es gibt aber keine lesbare Beschriftung, die das bestätigt.</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
@@ -5345,7 +5291,7 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>2026-10-23T23:41:43Z</t>
+          <t>2026-10-24T08:11:11Z</t>
         </is>
       </c>
     </row>
@@ -5375,12 +5321,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Bergkapelle Stoos (Maria Hilf Kapelle)</t>
+          <t>Bergkapelle Stoos</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Grosser Mythen; Kleiner Mythen</t>
+          <t>Gross Mythen; Chli Mythen</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -5397,7 +5343,7 @@
         <v>46.9804</v>
       </c>
       <c r="K48" t="n">
-        <v>8.664619999999999</v>
+        <v>8.664619</v>
       </c>
       <c r="L48" t="n">
         <v>2693275</v>
@@ -5406,26 +5352,26 @@
         <v>1203987</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="P48" s="3" t="n">
-        <v>0.85</v>
+        <v>0.962</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S48" s="3" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung); Gemeinde durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Geländeprüfung). In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
@@ -5440,7 +5386,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>Das amtliche Adressverzeichnis ordnet die Kapelle der Ortschaft Stoos SZ (6433) zu. | Das Gebäuderegister führt die Bergkapelle Stoos in der Ortschaft Stoos SZ. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190292528_0) | Die berechnete Silhouette vom Stoos mit Blick nach 23° zeigt die beiden Mythen genau an der Stelle wie auf dem Foto.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Die holzverschindelte Bergkapelle mit Dachreiter steht auf einem Hügel, und dahinter sieht man im Norden den Grossen und den Kleinen Mythen. Das passt zur Bergkapelle auf dem Stoos (Gemeinde Morschach).</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
@@ -5450,7 +5396,7 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>2026-10-23T23:42:49Z</t>
+          <t>2026-10-24T08:11:00Z</t>
         </is>
       </c>
     </row>
@@ -5468,69 +5414,37 @@
       <c r="C49" t="n">
         <v>1</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Wasserauen</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Berggasthaus Aescher-Wildkirchli</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Seealpsee; Alpstein; Ebenalp; Altmann</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Äscher 1</t>
-        </is>
-      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>09.07.2006</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>47.28336</v>
-      </c>
-      <c r="K49" t="n">
-        <v>9.414289999999999</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2749453</v>
-      </c>
-      <c r="M49" t="n">
-        <v>1238822</v>
-      </c>
       <c r="N49" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="O49" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P49" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="S49" s="3" t="n">
         <v>0</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Text im Bild, Session-Foto); Gemeinde nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Nicht im Kanton Schwyz: vermutlich Schwende-Rüte AI. Felder offen gelassen.</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Gemeinde</t>
+          <t>Ortschaft, Gemeinde, Gebäude, See/Fluss/Berg, Strasse</t>
         </is>
       </c>
       <c r="V49" s="4" t="inlineStr">
@@ -5543,11 +5457,6 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>Das Ortschaftenverzeichnis und das Adressverzeichnis ordnen den Punkt Äscher 1 der Ortschaft Wasserauen (PLZ 9057) in der Gemeinde Schwende-Rüte (AI) zu. | Der Schriftzug 'Aescher-Wildkirchli' am Gasthaus benennt den Ort oberhalb von Wasserauen. | Das Session-Foto zeigt die Wildkirchli-Höhle mit Kapelle direkt neben dem Gasthaus Aescher.</t>
-        </is>
-      </c>
       <c r="Y49" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -5555,7 +5464,7 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>2026-10-23T23:43:46Z</t>
+          <t>2026-10-24T08:11:00Z</t>
         </is>
       </c>
     </row>
@@ -5583,9 +5492,9 @@
           <t>Ingenbohl</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Gewerbegebäude Luzernerstrasse 22; Einstellhalle Gersauerstrasse 64; Gewerbegebäude Rubisacherweg 26</t>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Brunnen-Urmiberg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -5599,43 +5508,43 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>47.0009</v>
+        <v>47.001234</v>
       </c>
       <c r="K50" t="n">
-        <v>8.594900000000001</v>
+        <v>8.594244</v>
       </c>
       <c r="L50" t="n">
-        <v>2687937</v>
+        <v>2687887</v>
       </c>
       <c r="M50" t="n">
-        <v>1206186</v>
+        <v>1206222</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>0.95</v>
+        <v>0.962</v>
       </c>
       <c r="P50" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>0.7</v>
+        <v>0.962</v>
       </c>
       <c r="S50" s="3" t="n">
-        <v>1</v>
+        <v>0.962</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Ortschaft durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte, Session-Foto); Gemeinde durch 4 unabhängige Quellen gestützt (Gebäudeadressverzeichnis, Gebäuderegister (OSM/GWR), Karte, Session-Foto); See/Fluss/Berg nicht bestimmbar. In 2 unabhängigen Analysen übereinstimmend.</t>
+          <t>Stufe B: Zwei unabhängige Belege stimmen überein. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>See/Fluss/Berg</t>
+          <t>Gebäude</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
@@ -5650,7 +5559,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>Die amtliche Adresssuche an der Halle ergibt Ortschaft Brunnen (PLZ 6440). | Laut Gebäuderegister liegen die Gebäude Gersauerstrasse 64 und Rubisacherweg 26 in Brunnen. (https://api3.geo.admin.ch/rest/services/ech/MapServer/ch.bfs.gebaeude_wohnungs_register/190195709_0) | Das Luftbild SWISSIMAGE 2005 zeigt bei Wylen in Brunnen dieselbe Anordnung von Hallen, Wohnblöcken und Strasse.</t>
+          <t>Amtliches Register (GWR, OSM, KGS) am Ort des Motivs | 3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Auf den Hallen sind die Schriftzüge «SABAG» und «BOLFING AG» zu lesen. Die SABAG Brunnen hat ihren Sitz an der Luzernerstrasse 22 am Fuss des Urmibergs, und die Serie zeigt auch den Campingplatz an der Autobahn und die Muotamündung beim Hochwasser vom August 2005.</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
@@ -5660,7 +5569,7 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>2026-10-23T23:44:45Z</t>
+          <t>2026-10-24T08:11:13Z</t>
         </is>
       </c>
     </row>
@@ -5678,19 +5587,14 @@
       <c r="C51" t="n">
         <v>1</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Innerthal</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Innerthal</t>
-        </is>
-      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Wägitalersee; Fluebrig</t>
+          <t>Brünnelistock; Fluebrig; Rossalpelispitz; Wägitalersee; Zindlenspitz</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5699,43 +5603,43 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>47.099</v>
+        <v>47.090027</v>
       </c>
       <c r="K51" t="n">
-        <v>8.923999999999999</v>
+        <v>8.91826</v>
       </c>
       <c r="L51" t="n">
-        <v>2712757</v>
+        <v>2712340</v>
       </c>
       <c r="M51" t="n">
-        <v>1217511</v>
+        <v>1216505</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.95</v>
+        <v>0.571</v>
       </c>
       <c r="P51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>0.95</v>
+        <v>0.571</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S51" s="3" t="n">
-        <v>0.85</v>
+        <v>0.571</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>Ortschaft durch 3 unabhängigen Quellen gestützt (Gebäudeadressverzeichnis, swisstopo-Ortsname, Referenzfoto); Gemeinde durch 4 unabhängigen Quellen gestützt (Gebäudeadressverzeichnis, swisstopo-Ortsname, Referenzfoto, Bildinhalt); Gebäude, Strasse nicht bestimmbar.</t>
+          <t>Stufe C: Nur ein Beleg, meist Claudes Einschätzung des Bildes. Konfidenz: gemessene Trefferquote der Handprüfung.</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>Gebäude, Strasse</t>
+          <t>Ortschaft, Gebäude, Strasse</t>
         </is>
       </c>
       <c r="V51" s="4" t="inlineStr">
@@ -5750,7 +5654,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>Laut amtlichem Ortschaftenverzeichnis liegt der vermutete Standort am Ostufer des Wägitalersees in der Ortschaft Innerthal (PLZ 8858). | Laut swisstopo liegt der Wägitalersee in Innerthal. (https://api3.geo.admin.ch/rest/services/api/SearchServer?searchText=W%C3%A4gitalersee&amp;type=locations&amp;sr=2056&amp;limit=8) | Der ähnlichste Treffer zeigt den Stausee Innerthal mit gleicher Seeform und Bergkulisse (nicht verifiziert). (https://query.staatsarchiv.sz.ch/detail.aspx?ID=360234)</t>
+          <t>3 von 3 unabhängigen Untersuchungen nennen diese Gemeinde | Untersuchung 'all': Typischer grüner Stausee mit steilen Talflanken und Kalkgipfeln. Mit dem Referenzbild vom Wägitalersee stimmen dieselben Uferlinie, Alpweiden und Waldstücke überein. Blick vom Ufer bei Innerthal talaufwärts. | Untersuchung 'web': Ein grüner Stausee zwischen steilen Bergflanken mit den spitzen Kalkgipfeln im Süden, dazu ein Bild aus derselben Serie, das nach Norden Richtung Innerthal und Staumauer blickt: Das passt zum Ostufer des Wägitalersees.</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
@@ -5760,7 +5664,7 @@
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>2026-10-23T19:13:33Z</t>
+          <t>2026-10-24T08:11:02Z</t>
         </is>
       </c>
     </row>
@@ -7139,7 +7043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7161,144 +7065,120 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Konfidenz pro Feld</t>
+          <t>Ablauf</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Gezählt werden unabhängige Quellen, die den Wert stützen (verschiedene Art oder verschiedene Referenz). Der Wert stammt nicht aus einer Selbsteinschätzung des Modells.</t>
+          <t>1. Bildsuche über rund 52'000 Referenzfotos (Wikimedia Commons, Mapillary; MegaLoc, LightGlue). 2. Drei unabhängige Untersuchungen mit Claude (Opus 5.5): mit den Referenzfotos, ohne sie, und eine dritte ebenfalls nur mit dem Foto. Jede zoomt ins Original, liest Schrift, sucht im Web und in den amtlichen Registern (GWR, OSM, KGS-Inventar, swissNAMES3D) und nennt das Motiv mit seinem Registereintrag. 3. Ortschaft, Gemeinde, Strasse und Gebäude kommen aus dem Register am Ort des Motivs (nie vom Standort eines Vergleichsfotos). 4. Bildvergleich vor Ort: Fotos, die dort aufgenommen wurden (Mapillary, Wikimedia Commons), werden mit LightGlue geometrisch mit dem Foto verglichen. 5. Eine Schlussprüfung (Claude) sieht das Foto und alle Kandidaten mit ihren Vergleichsfotos, ohne zu wissen, wer sie vorgeschlagen hat, und wählt einen oder keinen.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>1 Quelle</t>
+          <t>Nicht bestimmbar</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>Ohne belastbaren Hinweis bleibt das Feld leer mit Konfidenz 0. Fotos ausserhalb des Kantons werden als solche markiert; leere Felder stehen in der Spalte Nicht_bestimmbar.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2 Quellen</t>
+          <t>Konfidenz</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>0.70</t>
+          <t>Stufe nach Regel, Zahl = gemessene Trefferquote der Stufe auf den von Hand geprüften Prio-1-Fotos (Gemeinde und Ortschaft richtig). Ohne Messung ein Schätzwert, das steht dann in Konfidenz_Begruendung.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3 Quellen</t>
+          <t>Prüfung nötig</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>ja, wenn die gemessene Konfidenz unter 0.90 liegt oder die Gemeinde fehlt. Nach einem Review (bestätigt oder korrigiert) nein; korrigierte Werte ersetzen die Vorschläge.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4 oder mehr Quellen</t>
+          <t>Stufe A</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>Bildvergleich vor Ort bestätigt, Gebäude bzw. Adresse im amtlichen Register, und mindestens zwei von drei unabhängigen Untersuchungen nennen dieselbe Gemeinde</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Gegenquelle</t>
+          <t>Stufe B</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Sagt eine echte Gegenquelle, dass der Wert falsch ist (verifiziertes Referenzfoto eines anderen Orts, Adressverzeichnis mit anderer Ortschaft oder Gemeinde, Text im Bild mit anderem Ort, verdeckte Sichtlinie), ist das Feld auf höchstens 0.60 begrenzt. Ein bloss möglicher anderer Kandidat ist keine Gegenquelle; er steht bei den verworfenen Hypothesen.</t>
+          <t>Zwei unabhängige Belege stimmen überein</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Nicht bestimmbar</t>
+          <t>Stufe C</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Ohne stützende Quelle bleibt das Feld leer und hat Konfidenz 0. Es wird nie ein Name geraten; leere Felder stehen in der Spalte Nicht_bestimmbar.</t>
+          <t>Nur ein Beleg, meist Claudes Einschätzung des Bildes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Konfidenz gesamt</t>
+          <t>Gemessen Stufe A</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Der tiefere Wert von Ortschaft und Gemeinde, plus 0.05, wenn auch Gebäude und Strasse bestimmt sind.</t>
+          <t>11 von 11 richtig, Konfidenz 0.92</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Konsistenzprüfung</t>
+          <t>Gemessen Stufe B</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Jedes Foto kann mehrmals unabhängig analysiert werden. Nennen die Analysen verschiedene Ortschaften oder Gemeinden, ist die Gesamtkonfidenz auf höchstens 0.60 begrenzt und eine Prüfung nötig; die Begründung nennt beide Orte.</t>
+          <t>24 von 24 richtig, Konfidenz 0.96</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Prüfung nötig</t>
+          <t>Gemessen Stufe C</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>ja, wenn die Gesamtkonfidenz unter 0.90 liegt, Ortschaft oder Gemeinde fehlt oder unabhängige Analysen verschiedene Orte nennen. Nach einem Review (bestätigt oder korrigiert) nein; korrigierte Werte ersetzen die Vorschläge der KI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Zählende Quellen</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Gebäudeadressverzeichnis (swisstopo), benanntes Gebäude aus OSM oder dem Gebäuderegister GWR, geometrisch verifiziertes Referenzfoto (LightGlue) aus Staatsarchiv / E-Pics / Smapshot / LUBIS / Wikimedia Commons, oder ein Referenzfoto mit bekanntem Aufnahmeort am vermuteten Ort, das dieselben Gebäude zeigt (ein nur ähnliches Foto zählt nicht), Archivdatensatz, swisstopo-Ortsname, Geländeprüfung (Sichtlinie oder Blickpunkt aus den sichtbaren Bergen), Text im Bild, Bildinhalt, Session-Foto (gleiche Kamera, unter 30 Minuten), EXIF-GPS. Werkzeug-Quellen zählen nur, wenn das Werkzeug in dieser Analyse wirklich aufgerufen wurde.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Einordnung</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Die Skala ist eine begründete Selbsteinschätzung, keine gemessene Trefferquote. Die gemessene Trefferquote pro Konfidenzstufe kommt aus einer von Hand geprüften Stichprobe.</t>
+          <t>3 von 5 richtig, Konfidenz 0.57</t>
         </is>
       </c>
     </row>

</xml_diff>